<commit_message>
updated BOM and added markdown file.
</commit_message>
<xml_diff>
--- a/versions/v0.9.2/BOM-v0.9.2.xlsx
+++ b/versions/v0.9.2/BOM-v0.9.2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asadiasm\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adowney2\Documents\GitHub\SEC-DAQ-Open-Source-Hardware-Design\versions\v0.9.2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8243814F-3B89-4E2E-A148-A74C8345F54F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EC4B306-3BB7-4791-B14A-67A5FB950CBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
+    <workbookView xWindow="-16320" yWindow="-6540" windowWidth="16440" windowHeight="28320" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
   <sheets>
     <sheet name="bill_of_materials" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="94">
   <si>
     <t>Total Cost</t>
   </si>
@@ -278,34 +278,46 @@
     <t>https://www.digikey.com/en/products/detail/everlight-electronics-co-ltd/EL3H7-TA-VG/2675689?s=N4IgTCBcDaIKIBkDMAJA7ACgCoEECUAtAGoDiIAugL5A</t>
   </si>
   <si>
-    <t>TDK</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/tdk/C1608X8R1E104M080AA/3951498?s=N4IgTCBcDaIMIEYBsAGAHADTQJQQUQRQBYBZdFAQQpAF0BfIA</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/tdk/C1608X7R1A105K080AC/2093406?s=N4IgTCBcDaIMIEYBsAGAHADQOwCUEEEEUBWAaXRXzhAF0BfIA</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/tdk/C1608X8R1E104K080AA/927126?s=N4IgTCBcDaIMIEYBsAGAHADTQJQQUQRQBYBpdFAQQoB1qQBdAXyA</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL10C510JB8NNNC/3887968?s=N4IgTCBcDaIMIBkCMAGOBWVApAQgDgDki4QBdAXyA</t>
-  </si>
-  <si>
-    <t>YAGEO</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/yageo/AC0603FR-07100RL/5895735?s=N4IgTCBcDaIIIGEAMA2JBmAYgJQLRIHYBGJJbAGRAF0BfIA</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/yageo/AC0603JR-0710KL/2827830?s=N4IgTCBcDaIIIGEAMA2JBmAUgJQLRIHYBGJAaQBkQBdAXyA</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/yageo/AC0603JR-074K7L/5896467?s=N4IgTCBcDaIIIGEAMA2JBmAUgJQLRIHYAWAaQIBkQBdAXyA</t>
-  </si>
-  <si>
     <t>order qty as needed</t>
+  </si>
+  <si>
+    <t>CAP CER 0.1UF 25V X8R 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/tdk/C1608X8R1E104M080AA/3951498</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/tdk/C1608X7R1A105K080AC/2093406</t>
+  </si>
+  <si>
+    <t>CAP CER 1UF 10V X7R 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/tdk/C1608X8R1E104K080AA/927126</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL10C510JB8NNNC/3887968</t>
+  </si>
+  <si>
+    <t>CAP CER 51PF 50V C0G/NP0 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/AC0603FR-07100RL/5895735</t>
+  </si>
+  <si>
+    <t>RES SMD 100 OHM 1% 1/10W 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/AC0603JR-0710KL/2827830</t>
+  </si>
+  <si>
+    <t>RES SMD 10K OHM 5% 1/10W 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/AC0603JR-074K7L/5896467</t>
+  </si>
+  <si>
+    <t>RES SMD 4.7K OHM 5% 1/10W 0603</t>
   </si>
 </sst>
 </file>
@@ -525,7 +537,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -726,15 +738,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -765,24 +768,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="13">
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -1069,6 +1054,24 @@
         </top>
       </border>
     </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1083,22 +1086,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3AC99790-742C-414B-AF83-048E0365A8B5}" name="Table1" displayName="Table1" ref="A1:K114" totalsRowShown="0" headerRowDxfId="0" tableBorderDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3AC99790-742C-414B-AF83-048E0365A8B5}" name="Table1" displayName="Table1" ref="A1:K114" totalsRowShown="0" headerRowDxfId="12" tableBorderDxfId="11">
   <autoFilter ref="A1:K114" xr:uid="{3AC99790-742C-414B-AF83-048E0365A8B5}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{7B25C464-EB0A-4B56-94DE-96F6AA8DEAC1}" name="Internal Part Name" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{DF8C1AF7-50DF-4DF9-864F-041981FCACF8}" name="MFR / Vendor Description" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{352F414F-9DAD-4EB9-9018-5EFFD7851FC0}" name="MFR Part Number" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{524EB195-1154-4033-90BB-70DCBC8C6954}" name="Quantity" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{16A43733-D0E2-469A-A9F1-7003745CBA03}" name="Individual Cost" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{5E3D3D1D-3CF3-463A-8FD2-F7FCD175AFB0}" name="Total Cost" dataDxfId="6">
+    <tableColumn id="1" xr3:uid="{7B25C464-EB0A-4B56-94DE-96F6AA8DEAC1}" name="Internal Part Name" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{DF8C1AF7-50DF-4DF9-864F-041981FCACF8}" name="MFR / Vendor Description" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{352F414F-9DAD-4EB9-9018-5EFFD7851FC0}" name="MFR Part Number" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{524EB195-1154-4033-90BB-70DCBC8C6954}" name="Quantity" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{16A43733-D0E2-469A-A9F1-7003745CBA03}" name="Individual Cost" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{5E3D3D1D-3CF3-463A-8FD2-F7FCD175AFB0}" name="Total Cost" dataDxfId="5">
       <calculatedColumnFormula>D2*E2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{75C60F91-0AB9-4643-82F8-4FD09187BCAB}" name="Notes" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{B2E8A010-1D06-4803-ADB8-641F00C3F533}" name="Vendor 1" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{C1A08220-EBF0-49C3-9563-C3B6645758E0}" name="Vendor 2" dataDxfId="3"/>
-    <tableColumn id="10" xr3:uid="{D3EFF0C9-98BD-4B48-90E8-5030DBC5DB99}" name="Vendor 3" dataDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{A06B68DA-A2F6-4D77-9FA7-22F7C10A75D6}" name="Vendor 4" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{75C60F91-0AB9-4643-82F8-4FD09187BCAB}" name="Notes" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{B2E8A010-1D06-4803-ADB8-641F00C3F533}" name="Vendor 1" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{C1A08220-EBF0-49C3-9563-C3B6645758E0}" name="Vendor 2" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{D3EFF0C9-98BD-4B48-90E8-5030DBC5DB99}" name="Vendor 3" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{A06B68DA-A2F6-4D77-9FA7-22F7C10A75D6}" name="Vendor 4" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1600,7 +1603,7 @@
       <c r="A8" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="74" t="s">
+      <c r="B8" s="17" t="s">
         <v>64</v>
       </c>
       <c r="C8" s="34" t="s">
@@ -1609,14 +1612,14 @@
       <c r="D8" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="80">
+      <c r="E8" s="77">
         <v>9.16</v>
       </c>
       <c r="F8" s="20" t="s">
         <v>30</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H8" s="36" t="s">
         <v>67</v>
@@ -1627,16 +1630,16 @@
       <c r="A9" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="75" t="s">
+      <c r="B9" s="10" t="s">
         <v>66</v>
       </c>
       <c r="C9" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="D9" s="77" t="s">
-        <v>30</v>
-      </c>
-      <c r="E9" s="81">
+      <c r="D9" s="74" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="78">
         <v>4.6399999999999997</v>
       </c>
       <c r="F9" s="12" t="s">
@@ -1654,7 +1657,7 @@
       <c r="A10" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="74" t="s">
+      <c r="B10" s="17" t="s">
         <v>69</v>
       </c>
       <c r="C10" s="34" t="s">
@@ -1663,7 +1666,7 @@
       <c r="D10" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="E10" s="80">
+      <c r="E10" s="77">
         <v>0.47</v>
       </c>
       <c r="F10" s="20" t="s">
@@ -1681,16 +1684,16 @@
       <c r="A11" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="75" t="s">
+      <c r="B11" s="10" t="s">
         <v>71</v>
       </c>
       <c r="C11" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="77" t="s">
-        <v>30</v>
-      </c>
-      <c r="E11" s="81">
+      <c r="D11" s="74" t="s">
+        <v>30</v>
+      </c>
+      <c r="E11" s="78">
         <v>2.54</v>
       </c>
       <c r="F11" s="12" t="s">
@@ -1705,7 +1708,7 @@
       <c r="A12" s="33" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="74" t="s">
+      <c r="B12" s="17" t="s">
         <v>73</v>
       </c>
       <c r="C12" s="34" t="s">
@@ -1730,16 +1733,16 @@
       <c r="A13" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="75" t="s">
+      <c r="B13" s="10" t="s">
         <v>73</v>
       </c>
       <c r="C13" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="D13" s="77" t="s">
-        <v>30</v>
-      </c>
-      <c r="E13" s="82">
+      <c r="D13" s="74" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" s="79">
         <v>1.64</v>
       </c>
       <c r="F13" s="12" t="s">
@@ -1755,7 +1758,7 @@
       <c r="A14" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="74" t="s">
+      <c r="B14" s="17" t="s">
         <v>76</v>
       </c>
       <c r="C14" s="33" t="s">
@@ -1780,16 +1783,16 @@
       <c r="A15" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="75" t="s">
+      <c r="B15" s="10" t="s">
         <v>78</v>
       </c>
       <c r="C15" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="D15" s="77" t="s">
-        <v>30</v>
-      </c>
-      <c r="E15" s="81">
+      <c r="D15" s="74" t="s">
+        <v>30</v>
+      </c>
+      <c r="E15" s="78">
         <v>0.51</v>
       </c>
       <c r="F15" s="12" t="s">
@@ -1818,7 +1821,7 @@
         <v>48</v>
       </c>
       <c r="C17" s="45"/>
-      <c r="D17" s="77"/>
+      <c r="D17" s="74"/>
       <c r="E17" s="2"/>
       <c r="F17" s="12"/>
       <c r="G17" s="25"/>
@@ -1829,8 +1832,8 @@
       <c r="A18" s="33" t="s">
         <v>50</v>
       </c>
-      <c r="B18" s="74" t="s">
-        <v>80</v>
+      <c r="B18" s="17" t="s">
+        <v>81</v>
       </c>
       <c r="C18" s="33" t="s">
         <v>57</v>
@@ -1846,7 +1849,7 @@
       </c>
       <c r="G18" s="21"/>
       <c r="H18" s="22" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I18" s="23"/>
     </row>
@@ -1854,13 +1857,13 @@
       <c r="A19" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="B19" s="75" t="s">
-        <v>80</v>
+      <c r="B19" s="10" t="s">
+        <v>84</v>
       </c>
       <c r="C19" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="D19" s="77" t="s">
+      <c r="D19" s="74" t="s">
         <v>30</v>
       </c>
       <c r="E19" s="11">
@@ -1870,8 +1873,8 @@
         <v>30</v>
       </c>
       <c r="G19" s="25"/>
-      <c r="H19" s="9" t="s">
-        <v>82</v>
+      <c r="H19" s="14" t="s">
+        <v>83</v>
       </c>
       <c r="I19" s="32"/>
     </row>
@@ -1879,8 +1882,8 @@
       <c r="A20" s="33" t="s">
         <v>50</v>
       </c>
-      <c r="B20" s="74" t="s">
-        <v>80</v>
+      <c r="B20" s="17" t="s">
+        <v>81</v>
       </c>
       <c r="C20" s="33" t="s">
         <v>60</v>
@@ -1896,7 +1899,7 @@
       </c>
       <c r="G20" s="21"/>
       <c r="H20" s="22" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I20" s="23"/>
     </row>
@@ -1904,13 +1907,13 @@
       <c r="A21" s="28" t="s">
         <v>51</v>
       </c>
-      <c r="B21" s="75" t="s">
-        <v>80</v>
+      <c r="B21" s="10" t="s">
+        <v>87</v>
       </c>
       <c r="C21" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="D21" s="77" t="s">
+      <c r="D21" s="74" t="s">
         <v>30</v>
       </c>
       <c r="E21" s="11">
@@ -1921,7 +1924,7 @@
       </c>
       <c r="G21" s="25"/>
       <c r="H21" s="14" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I21" s="32"/>
     </row>
@@ -1938,11 +1941,11 @@
     </row>
     <row r="23" spans="1:9" s="13" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="43"/>
-      <c r="B23" s="78" t="s">
+      <c r="B23" s="75" t="s">
         <v>52</v>
       </c>
       <c r="C23" s="43"/>
-      <c r="D23" s="79"/>
+      <c r="D23" s="76"/>
       <c r="E23" s="38"/>
       <c r="F23" s="12"/>
       <c r="G23" s="25"/>
@@ -1953,24 +1956,24 @@
       <c r="A24" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B24" s="76" t="s">
-        <v>85</v>
+      <c r="B24" s="50" t="s">
+        <v>89</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D24" s="77" t="s">
+      <c r="D24" s="74" t="s">
         <v>30</v>
       </c>
       <c r="E24" s="11">
         <v>0.1</v>
       </c>
-      <c r="F24" s="84" t="s">
+      <c r="F24" s="81" t="s">
         <v>30</v>
       </c>
       <c r="G24" s="5"/>
       <c r="H24" s="14" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I24" s="53"/>
     </row>
@@ -1978,8 +1981,8 @@
       <c r="A25" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B25" s="76" t="s">
-        <v>85</v>
+      <c r="B25" s="50" t="s">
+        <v>91</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>62</v>
@@ -1987,15 +1990,15 @@
       <c r="D25" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="E25" s="83">
+      <c r="E25" s="80">
         <v>0.1</v>
       </c>
-      <c r="F25" s="84" t="s">
+      <c r="F25" s="81" t="s">
         <v>30</v>
       </c>
       <c r="G25" s="3"/>
       <c r="H25" s="52" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="I25" s="53"/>
     </row>
@@ -2003,24 +2006,24 @@
       <c r="A26" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B26" s="76" t="s">
-        <v>85</v>
+      <c r="B26" s="50" t="s">
+        <v>93</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D26" s="77" t="s">
+      <c r="D26" s="74" t="s">
         <v>30</v>
       </c>
       <c r="E26" s="11">
         <v>0.1</v>
       </c>
-      <c r="F26" s="84" t="s">
+      <c r="F26" s="81" t="s">
         <v>30</v>
       </c>
       <c r="G26" s="3"/>
       <c r="H26" s="14" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="I26" s="3"/>
     </row>

</xml_diff>